<commit_message>
Results: Orange County rerun — 958/1100 fields, identity audit clean
Full Set3 rerun with the Orange County fixes (b89e715):

- Coverage 948 -> 958/1100 (87.1%); 55 files now complete (11/11)
- Orange County 0/11 -> 10/11; its four captured FB categories sum to
  the reported total exactly (committed genuinely absent)
- Zero-extraction bucket down to 2 (Arkansas, Atlanta — OCR cases)
- Only other change: NY State's BS page is now FOUND (explicit NOT
  FOUNDs instead of silent absence; rotated-text extraction still on
  the backlog)
- Identity audit: 0 findings across all 113 files (FB identity 78/78)
- Regression gate 12: Set1 8/8 + Set2 5/5 identical

Backup snapshot refreshed (script sha256-verified); CLAUDE.md state
and backlog updated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Backups/2026-07-07_audited/FY25_Set3_results.xlsx
+++ b/Backups/2026-07-07_audited/FY25_Set3_results.xlsx
@@ -1697,123 +1697,83 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Full Dollars</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+          <t>Thousands</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>2087077</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>455452</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>2324</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>184685</v>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="L13" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="M13" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N13" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="O13" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="J13" s="4" t="n">
+        <v>31447</v>
+      </c>
+      <c r="K13" s="4" t="n">
+        <v>1221849</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>1440305</v>
+      </c>
+      <c r="M13" s="4" t="n">
+        <v>4391867</v>
+      </c>
+      <c r="N13" s="4" t="n">
+        <v>4685192</v>
+      </c>
+      <c r="O13" s="4" t="n">
+        <v>445058</v>
       </c>
       <c r="P13" s="5" t="inlineStr">
         <is>
-          <t>BS p41: General Fund column not identified | RevEx p41: General Fund column not identified</t>
-        </is>
-      </c>
-      <c r="Q13" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="R13" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="S13" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="T13" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+          <t>BS: spread layout — General Fund column on facing page 66 | NOT FOUND: committed | RevEx: spread layout — General Fund column on facing page 70</t>
+        </is>
+      </c>
+      <c r="Q13" s="4" t="n">
+        <v>2087077000</v>
+      </c>
+      <c r="R13" s="4" t="n">
+        <v>455452000</v>
+      </c>
+      <c r="S13" s="4" t="n">
+        <v>2324000</v>
+      </c>
+      <c r="T13" s="4" t="n">
+        <v>184685000</v>
       </c>
       <c r="U13" s="6" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="V13" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="W13" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="X13" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Y13" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z13" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="AA13" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="V13" s="4" t="n">
+        <v>31447000</v>
+      </c>
+      <c r="W13" s="4" t="n">
+        <v>1221849000</v>
+      </c>
+      <c r="X13" s="4" t="n">
+        <v>1440305000</v>
+      </c>
+      <c r="Y13" s="4" t="n">
+        <v>4391867000</v>
+      </c>
+      <c r="Z13" s="4" t="n">
+        <v>4685192000</v>
+      </c>
+      <c r="AA13" s="4" t="n">
+        <v>445058000</v>
       </c>
     </row>
     <row r="14">
@@ -7423,7 +7383,7 @@
       </c>
       <c r="P71" s="5" t="inlineStr">
         <is>
-          <t>Unit disclosure differs between statement pages: {16: 'Full Dollars', 43: 'Millions'} — verify normalized figures manually | BS p17: General Fund column not identified | NOT FOUND: total_ofs</t>
+          <t>Unit disclosure differs between statement pages: {16: 'Full Dollars', 43: 'Millions'} — verify normalized figures manually | BS: spread layout — General Fund column on facing page 16 | NOT FOUND: total_assets | NOT FOUND: total_liabilities | NOT FOUND: nonspendable | NOT FOUND: restricted | NOT FOUND: committed | NOT FOUND: assigned | NOT FOUND: unassigned | NOT FOUND: total_fund_balances | NOT FOUND: total_ofs</t>
         </is>
       </c>
       <c r="Q71" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Results: OCR run — 979/1100 fields (89.0%), zero-extraction bucket empty
Full Set3 rerun with the OCR layer:

- Coverage 958 -> 979/1100; 56 files complete (11/11); ZERO files at 0/11
  for the first time (was 5 at campaign start)
- Arkansas 0/11 -> 11/11 (expenditures derived from excess line, noted);
  Atlanta 0/11 -> 10/11 (OFS still missing — backlog)
- Both files' FB categories sum to their reported totals exactly —
  tesseract digit accuracy verified by identity
- All 22 changed cells vs prior run are Arkansas/Atlanta; the six files
  regressed by the interim global tolerance are fully restored
- Identity audit: 0 findings, FB identity 80/80 across all three sets
- Backup snapshot refreshed (script sha256-verified); CLAUDE.md updated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Backups/2026-07-07_audited/FY25_Set3_results.xlsx
+++ b/Backups/2026-07-07_audited/FY25_Set3_results.xlsx
@@ -899,133 +899,89 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>State of Arkansas</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>June 30, 2025</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="I5" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N5" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="O5" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+          <t>Thousands</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>14098287</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>1745641</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>141847</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>2440372</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>8769047</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>47633</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>74161</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>11473060</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>24769923</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>23098631</v>
+      </c>
+      <c r="O5" s="4" t="n">
+        <v>-766977</v>
       </c>
       <c r="P5" s="5" t="inlineStr">
         <is>
-          <t>Text layer unusable (broken font encoding) — needs OCR; skipped full scan</t>
-        </is>
-      </c>
-      <c r="Q5" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="R5" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="S5" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="T5" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="U5" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="V5" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="W5" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="X5" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Y5" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z5" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="AA5" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+          <t>Text layer unusable — figures extracted via OCR; verify manually | Total expenditures derived from excess line (revenues - excess) — value row unreadable</t>
+        </is>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>14098287000</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <v>1745641000</v>
+      </c>
+      <c r="S5" s="4" t="n">
+        <v>141847000</v>
+      </c>
+      <c r="T5" s="4" t="n">
+        <v>2440372000</v>
+      </c>
+      <c r="U5" s="4" t="n">
+        <v>8769047000</v>
+      </c>
+      <c r="V5" s="4" t="n">
+        <v>47633000</v>
+      </c>
+      <c r="W5" s="4" t="n">
+        <v>74161000</v>
+      </c>
+      <c r="X5" s="4" t="n">
+        <v>11473060000</v>
+      </c>
+      <c r="Y5" s="4" t="n">
+        <v>24769923000</v>
+      </c>
+      <c r="Z5" s="4" t="n">
+        <v>23098631000</v>
+      </c>
+      <c r="AA5" s="4" t="n">
+        <v>-766977000</v>
       </c>
     </row>
     <row r="6">
@@ -3134,68 +3090,48 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>City of Atlanta</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
+          <t>June 30, 2025</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="J28" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="K28" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="L28" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="M28" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N28" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+          <t>Thousands</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>272412</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>52682</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>61713</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>1201</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>14481</v>
+      </c>
+      <c r="K28" s="4" t="n">
+        <v>127695</v>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>205090</v>
+      </c>
+      <c r="M28" s="4" t="n">
+        <v>833798</v>
+      </c>
+      <c r="N28" s="4" t="n">
+        <v>874567</v>
       </c>
       <c r="O28" s="3" t="inlineStr">
         <is>
@@ -3204,58 +3140,38 @@
       </c>
       <c r="P28" s="5" t="inlineStr">
         <is>
-          <t>Text layer unusable (broken font encoding) — needs OCR; skipped full scan</t>
-        </is>
-      </c>
-      <c r="Q28" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="R28" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="S28" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="T28" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="U28" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="V28" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="W28" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="X28" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Y28" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z28" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+          <t>Text layer unusable — figures extracted via OCR; verify manually | NOT FOUND: total_ofs</t>
+        </is>
+      </c>
+      <c r="Q28" s="4" t="n">
+        <v>272412000</v>
+      </c>
+      <c r="R28" s="4" t="n">
+        <v>52682000</v>
+      </c>
+      <c r="S28" s="4" t="n">
+        <v>61713000</v>
+      </c>
+      <c r="T28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U28" s="4" t="n">
+        <v>1201000</v>
+      </c>
+      <c r="V28" s="4" t="n">
+        <v>14481000</v>
+      </c>
+      <c r="W28" s="4" t="n">
+        <v>127695000</v>
+      </c>
+      <c r="X28" s="4" t="n">
+        <v>205090000</v>
+      </c>
+      <c r="Y28" s="4" t="n">
+        <v>833798000</v>
+      </c>
+      <c r="Z28" s="4" t="n">
+        <v>874567000</v>
       </c>
       <c r="AA28" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Results: per-page OCR run — 983/1100 (89.4%), identity audit clean
Final Set3 run with the per-page OCR fallbacks (c8ca62f) plus the
rev/exp plausibility gate on OCR adoption:

- Coverage 979 -> 983/1100; changed cells are exactly the four expected
  gains (Allegheny RevEx totals, Massachusetts RevEx totals) — zero
  collateral movement
- San Antonio BS gains live on the Set1 side (0 -> 8 fields, cross-
  verified against its native RevEx ending fund balance)
- Honolulu's implausible OCR adoption (rev/exp ratio 0.01, caught by
  the identity audit) is gated out — reverted to honest NOT FOUNDs
- Identity audit: 0 findings, FB identity 81/81 across all three sets
- Backup snapshot refreshed (sha256-verified); CLAUDE.md updated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Backups/2026-07-07_audited/FY25_Set3_results.xlsx
+++ b/Backups/2026-07-07_audited/FY25_Set3_results.xlsx
@@ -4800,22 +4800,18 @@
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M45" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N45" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="M45" s="4" t="n">
+        <v>61907573</v>
+      </c>
+      <c r="N45" s="4" t="n">
+        <v>58604191</v>
       </c>
       <c r="O45" s="4" t="n">
         <v>2650066</v>
       </c>
       <c r="P45" s="5" t="inlineStr">
         <is>
-          <t>BS p55: continuation carries other funds — page skipped | NOT FOUND: nonspendable | NOT FOUND: total_fund_balances | NOT FOUND: total_revenues | NOT FOUND: total_expenditures</t>
+          <t>BS p55: continuation carries other funds — page skipped | NOT FOUND: nonspendable | NOT FOUND: total_fund_balances | RevEx re-extracted via OCR (native value zone unreadable) — verify manually</t>
         </is>
       </c>
       <c r="Q45" s="4" t="n">
@@ -4846,15 +4842,11 @@
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y45" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z45" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="Y45" s="4" t="n">
+        <v>61907573000</v>
+      </c>
+      <c r="Z45" s="4" t="n">
+        <v>58604191000</v>
       </c>
       <c r="AA45" s="4" t="n">
         <v>2650066000</v>
@@ -7896,15 +7888,11 @@
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="M77" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N77" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="M77" s="4" t="n">
+        <v>1018984833</v>
+      </c>
+      <c r="N77" s="4" t="n">
+        <v>976221125</v>
       </c>
       <c r="O77" s="3" t="inlineStr">
         <is>
@@ -7913,7 +7901,7 @@
       </c>
       <c r="P77" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: nonspendable | NOT FOUND: restricted | NOT FOUND: committed | NOT FOUND: assigned | NOT FOUND: unassigned | NOT FOUND: total_fund_balances | NOT FOUND: total_revenues | NOT FOUND: total_expenditures | NOT FOUND: total_ofs</t>
+          <t>NOT FOUND: nonspendable | NOT FOUND: restricted | NOT FOUND: committed | NOT FOUND: assigned | NOT FOUND: unassigned | NOT FOUND: total_fund_balances | RevEx re-extracted via OCR (native value zone unreadable) — verify manually | NOT FOUND: total_ofs</t>
         </is>
       </c>
       <c r="Q77" s="4" t="n">
@@ -7952,15 +7940,11 @@
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="Y77" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z77" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="Y77" s="4" t="n">
+        <v>1018984833</v>
+      </c>
+      <c r="Z77" s="4" t="n">
+        <v>976221125</v>
       </c>
       <c r="AA77" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Results: triage wave — 1033/1100 fields (93.9%), identity audit clean
Full Set3 rerun after the 9-fix triage wave (see prior commit):

- Coverage 983 -> 1033/1100; 56 gains vs 6 losses (all six are the
  None->0.0 honesty conversion on unverifiable category zeros)
- 7 bonus gains outside the diagnosed files (San Diego County, Georgia,
  Polk, Minnesota, Pennsylvania, South Dakota) from the title anchors
  and the net-other-financing OFS pattern
- Both silent-wrong values verified corrected in the workbook
- Identity audit: 0 findings, FB identity 78/78 across all three sets
- Backup refreshed (sha256-verified); CLAUDE.md updated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Backups/2026-07-07_audited/FY25_Set3_results.xlsx
+++ b/Backups/2026-07-07_audited/FY25_Set3_results.xlsx
@@ -1208,11 +1208,15 @@
       <c r="G8" s="4" t="n">
         <v>7002446</v>
       </c>
-      <c r="H8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>0</v>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
       </c>
       <c r="J8" s="4" t="n">
         <v>358489153</v>
@@ -1232,7 +1236,11 @@
       <c r="O8" s="4" t="n">
         <v>-515904125</v>
       </c>
-      <c r="P8" s="5" t="inlineStr"/>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>NOT FOUND: restricted | NOT FOUND: committed</t>
+        </is>
+      </c>
       <c r="Q8" s="4" t="n">
         <v>508420528</v>
       </c>
@@ -1242,11 +1250,15 @@
       <c r="S8" s="4" t="n">
         <v>7002446</v>
       </c>
-      <c r="T8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U8" s="4" t="n">
-        <v>0</v>
+      <c r="T8" s="6" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U8" s="6" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
       </c>
       <c r="V8" s="4" t="n">
         <v>358489153</v>
@@ -1299,8 +1311,10 @@
       <c r="G9" s="4" t="n">
         <v>2851</v>
       </c>
-      <c r="H9" s="4" t="n">
-        <v>0</v>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
       </c>
       <c r="I9" s="4" t="n">
         <v>122044</v>
@@ -1325,7 +1339,7 @@
       </c>
       <c r="P9" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: total_liabilities</t>
+          <t>NOT FOUND: total_liabilities | NOT FOUND: restricted</t>
         </is>
       </c>
       <c r="Q9" s="4" t="n">
@@ -1339,8 +1353,10 @@
       <c r="S9" s="4" t="n">
         <v>2851000</v>
       </c>
-      <c r="T9" s="4" t="n">
-        <v>0</v>
+      <c r="T9" s="6" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
       </c>
       <c r="U9" s="4" t="n">
         <v>122044000</v>
@@ -1418,11 +1434,7 @@
       <c r="O10" s="4" t="n">
         <v>-9512</v>
       </c>
-      <c r="P10" s="5" t="inlineStr">
-        <is>
-          <t>BS page 61 inferred by position (title unreadable) — verify manually</t>
-        </is>
-      </c>
+      <c r="P10" s="5" t="inlineStr"/>
       <c r="Q10" s="4" t="n">
         <v>191367000</v>
       </c>
@@ -1866,24 +1878,16 @@
       <c r="L15" s="4" t="n">
         <v>3045454</v>
       </c>
-      <c r="M15" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="M15" s="4" t="n">
+        <v>6068285</v>
       </c>
       <c r="N15" s="4" t="n">
         <v>6195665</v>
       </c>
-      <c r="O15" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="P15" s="5" t="inlineStr">
-        <is>
-          <t>NOT FOUND: total_revenues | NOT FOUND: total_ofs</t>
-        </is>
-      </c>
+      <c r="O15" s="4" t="n">
+        <v>179904</v>
+      </c>
+      <c r="P15" s="5" t="inlineStr"/>
       <c r="Q15" s="4" t="n">
         <v>4553571000</v>
       </c>
@@ -1908,18 +1912,14 @@
       <c r="X15" s="4" t="n">
         <v>3045454000</v>
       </c>
-      <c r="Y15" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="Y15" s="4" t="n">
+        <v>6068285000</v>
       </c>
       <c r="Z15" s="4" t="n">
         <v>6195665000</v>
       </c>
-      <c r="AA15" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="AA15" s="4" t="n">
+        <v>179904000</v>
       </c>
     </row>
     <row r="16">
@@ -2145,26 +2145,16 @@
       <c r="L18" s="4" t="n">
         <v>3786963</v>
       </c>
-      <c r="M18" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N18" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="O18" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="P18" s="5" t="inlineStr">
-        <is>
-          <t>RevEx p53: General Fund column not identified</t>
-        </is>
-      </c>
+      <c r="M18" s="4" t="n">
+        <v>27950701</v>
+      </c>
+      <c r="N18" s="4" t="n">
+        <v>27559901</v>
+      </c>
+      <c r="O18" s="4" t="n">
+        <v>-516252</v>
+      </c>
+      <c r="P18" s="5" t="inlineStr"/>
       <c r="Q18" s="4" t="n">
         <v>8982837000</v>
       </c>
@@ -2189,20 +2179,14 @@
       <c r="X18" s="4" t="n">
         <v>3786963000</v>
       </c>
-      <c r="Y18" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z18" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="AA18" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="Y18" s="4" t="n">
+        <v>27950701000</v>
+      </c>
+      <c r="Z18" s="4" t="n">
+        <v>27559901000</v>
+      </c>
+      <c r="AA18" s="4" t="n">
+        <v>-516252000</v>
       </c>
     </row>
     <row r="19">
@@ -2768,24 +2752,20 @@
           <t>Thousands</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="E25" s="4" t="n">
+        <v>1078636</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>224317</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0</v>
+        <v>29366</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>0</v>
+        <v>114955</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>0</v>
+        <v>124286</v>
       </c>
       <c r="J25" s="4" t="n">
         <v>321723</v>
@@ -2793,49 +2773,33 @@
       <c r="K25" s="4" t="n">
         <v>225803</v>
       </c>
-      <c r="L25" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="M25" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N25" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="O25" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="P25" s="5" t="inlineStr">
-        <is>
-          <t>BS page 60 inferred by position (title unreadable) — verify manually | NOT FOUND: total_assets | NOT FOUND: total_liabilities | NOT FOUND: total_fund_balances | NOT FOUND: total_revenues | NOT FOUND: total_expenditures | NOT FOUND: total_ofs</t>
-        </is>
-      </c>
-      <c r="Q25" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="R25" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="L25" s="4" t="n">
+        <v>816133</v>
+      </c>
+      <c r="M25" s="4" t="n">
+        <v>3858839</v>
+      </c>
+      <c r="N25" s="4" t="n">
+        <v>3080641</v>
+      </c>
+      <c r="O25" s="4" t="n">
+        <v>-780362</v>
+      </c>
+      <c r="P25" s="5" t="inlineStr"/>
+      <c r="Q25" s="4" t="n">
+        <v>1078636000</v>
+      </c>
+      <c r="R25" s="4" t="n">
+        <v>224317000</v>
       </c>
       <c r="S25" s="4" t="n">
-        <v>0</v>
+        <v>29366000</v>
       </c>
       <c r="T25" s="4" t="n">
-        <v>0</v>
+        <v>114955000</v>
       </c>
       <c r="U25" s="4" t="n">
-        <v>0</v>
+        <v>124286000</v>
       </c>
       <c r="V25" s="4" t="n">
         <v>321723000</v>
@@ -2843,25 +2807,17 @@
       <c r="W25" s="4" t="n">
         <v>225803000</v>
       </c>
-      <c r="X25" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Y25" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z25" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="AA25" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="X25" s="4" t="n">
+        <v>816133000</v>
+      </c>
+      <c r="Y25" s="4" t="n">
+        <v>3858839000</v>
+      </c>
+      <c r="Z25" s="4" t="n">
+        <v>3080641000</v>
+      </c>
+      <c r="AA25" s="4" t="n">
+        <v>-780362000</v>
       </c>
     </row>
     <row r="26">
@@ -2911,24 +2867,18 @@
       <c r="L26" s="4" t="n">
         <v>572036380</v>
       </c>
-      <c r="M26" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N26" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="O26" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="M26" s="4" t="n">
+        <v>2013797873</v>
+      </c>
+      <c r="N26" s="4" t="n">
+        <v>1731292993</v>
+      </c>
+      <c r="O26" s="4" t="n">
+        <v>-294238420</v>
       </c>
       <c r="P26" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: committed | RevEx p41: General Fund column not identified</t>
+          <t>NOT FOUND: committed</t>
         </is>
       </c>
       <c r="Q26" s="4" t="n">
@@ -2957,20 +2907,14 @@
       <c r="X26" s="4" t="n">
         <v>572036380</v>
       </c>
-      <c r="Y26" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z26" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="AA26" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="Y26" s="4" t="n">
+        <v>2013797873</v>
+      </c>
+      <c r="Z26" s="4" t="n">
+        <v>1731292993</v>
+      </c>
+      <c r="AA26" s="4" t="n">
+        <v>-294238420</v>
       </c>
     </row>
     <row r="27">
@@ -3020,24 +2964,18 @@
       <c r="L27" s="4" t="n">
         <v>31207660</v>
       </c>
-      <c r="M27" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N27" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="O27" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="M27" s="4" t="n">
+        <v>59180534</v>
+      </c>
+      <c r="N27" s="4" t="n">
+        <v>54768079</v>
+      </c>
+      <c r="O27" s="4" t="n">
+        <v>-5416022</v>
       </c>
       <c r="P27" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: assigned | NOT FOUND: total_revenues | NOT FOUND: total_expenditures | NOT FOUND: total_ofs</t>
+          <t>NOT FOUND: assigned</t>
         </is>
       </c>
       <c r="Q27" s="4" t="n">
@@ -3066,20 +3004,14 @@
       <c r="X27" s="4" t="n">
         <v>31207660000</v>
       </c>
-      <c r="Y27" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z27" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="AA27" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="Y27" s="4" t="n">
+        <v>59180534000</v>
+      </c>
+      <c r="Z27" s="4" t="n">
+        <v>54768079000</v>
+      </c>
+      <c r="AA27" s="4" t="n">
+        <v>-5416022000</v>
       </c>
     </row>
     <row r="28">
@@ -3140,7 +3072,7 @@
       </c>
       <c r="P28" s="5" t="inlineStr">
         <is>
-          <t>Text layer unusable — figures extracted via OCR; verify manually | NOT FOUND: total_ofs</t>
+          <t>Text layer unusable — figures extracted via OCR; verify manually | RevEx page 61 inferred by position (title unreadable) — verify manually | NOT FOUND: total_ofs</t>
         </is>
       </c>
       <c r="Q28" s="4" t="n">
@@ -3230,16 +3162,10 @@
       <c r="N29" s="4" t="n">
         <v>62533774</v>
       </c>
-      <c r="O29" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="P29" s="5" t="inlineStr">
-        <is>
-          <t>NOT FOUND: total_ofs</t>
-        </is>
-      </c>
+      <c r="O29" s="4" t="n">
+        <v>-7574043</v>
+      </c>
+      <c r="P29" s="5" t="inlineStr"/>
       <c r="Q29" s="4" t="n">
         <v>36450272000</v>
       </c>
@@ -3270,10 +3196,8 @@
       <c r="Z29" s="4" t="n">
         <v>62533774000</v>
       </c>
-      <c r="AA29" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="AA29" s="4" t="n">
+        <v>-7574043000</v>
       </c>
     </row>
     <row r="30">
@@ -3451,7 +3375,7 @@
       </c>
       <c r="P31" s="5" t="inlineStr">
         <is>
-          <t>BS page 41 inferred by position (title unreadable) — verify manually | NOT FOUND: nonspendable | OFS total found via positional fallback (label non-standard)</t>
+          <t>NOT FOUND: nonspendable | OFS total found via positional fallback (label non-standard)</t>
         </is>
       </c>
       <c r="Q31" s="4" t="n">
@@ -3537,22 +3461,18 @@
       <c r="L32" s="4" t="n">
         <v>178618913</v>
       </c>
-      <c r="M32" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N32" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="M32" s="4" t="n">
+        <v>253351989</v>
+      </c>
+      <c r="N32" s="4" t="n">
+        <v>285877401</v>
       </c>
       <c r="O32" s="4" t="n">
         <v>4424284</v>
       </c>
       <c r="P32" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: assigned | NOT FOUND: total_revenues | NOT FOUND: total_expenditures</t>
+          <t>NOT FOUND: assigned</t>
         </is>
       </c>
       <c r="Q32" s="4" t="n">
@@ -3581,15 +3501,11 @@
       <c r="X32" s="4" t="n">
         <v>178618913</v>
       </c>
-      <c r="Y32" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z32" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="Y32" s="4" t="n">
+        <v>253351989</v>
+      </c>
+      <c r="Z32" s="4" t="n">
+        <v>285877401</v>
       </c>
       <c r="AA32" s="4" t="n">
         <v>4424284</v>
@@ -4421,11 +4337,7 @@
       <c r="O41" s="4" t="n">
         <v>-98995629</v>
       </c>
-      <c r="P41" s="5" t="inlineStr">
-        <is>
-          <t>BS page 38 inferred by position (title unreadable) — verify manually</t>
-        </is>
-      </c>
+      <c r="P41" s="5" t="inlineStr"/>
       <c r="Q41" s="4" t="n">
         <v>301157079</v>
       </c>
@@ -4490,8 +4402,10 @@
       <c r="G42" s="4" t="n">
         <v>6485</v>
       </c>
-      <c r="H42" s="4" t="n">
-        <v>0</v>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
       </c>
       <c r="I42" s="4" t="n">
         <v>0</v>
@@ -4505,24 +4419,18 @@
       <c r="L42" s="4" t="n">
         <v>6432440</v>
       </c>
-      <c r="M42" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N42" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="O42" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="M42" s="4" t="n">
+        <v>15541675</v>
+      </c>
+      <c r="N42" s="4" t="n">
+        <v>14495976</v>
+      </c>
+      <c r="O42" s="4" t="n">
+        <v>-1320063</v>
       </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: total_revenues | NOT FOUND: total_expenditures | NOT FOUND: total_ofs</t>
+          <t>NOT FOUND: restricted</t>
         </is>
       </c>
       <c r="Q42" s="4" t="n">
@@ -4534,8 +4442,10 @@
       <c r="S42" s="4" t="n">
         <v>6485000</v>
       </c>
-      <c r="T42" s="4" t="n">
-        <v>0</v>
+      <c r="T42" s="6" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
       </c>
       <c r="U42" s="4" t="n">
         <v>0</v>
@@ -4549,20 +4459,14 @@
       <c r="X42" s="4" t="n">
         <v>6432440000</v>
       </c>
-      <c r="Y42" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z42" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="AA42" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="Y42" s="4" t="n">
+        <v>15541675000</v>
+      </c>
+      <c r="Z42" s="4" t="n">
+        <v>14495976000</v>
+      </c>
+      <c r="AA42" s="4" t="n">
+        <v>-1320063000</v>
       </c>
     </row>
     <row r="43">
@@ -4899,24 +4803,18 @@
       <c r="L46" s="4" t="n">
         <v>923828</v>
       </c>
-      <c r="M46" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N46" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="O46" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="M46" s="4" t="n">
+        <v>2521134</v>
+      </c>
+      <c r="N46" s="4" t="n">
+        <v>2448826</v>
+      </c>
+      <c r="O46" s="4" t="n">
+        <v>-70543</v>
       </c>
       <c r="P46" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: committed | RevEx p37: General Fund column not identified</t>
+          <t>NOT FOUND: committed</t>
         </is>
       </c>
       <c r="Q46" s="4" t="n">
@@ -4945,20 +4843,14 @@
       <c r="X46" s="4" t="n">
         <v>923828000</v>
       </c>
-      <c r="Y46" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z46" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="AA46" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="Y46" s="4" t="n">
+        <v>2521134000</v>
+      </c>
+      <c r="Z46" s="4" t="n">
+        <v>2448826000</v>
+      </c>
+      <c r="AA46" s="4" t="n">
+        <v>-70543000</v>
       </c>
     </row>
     <row r="47">
@@ -5294,7 +5186,11 @@
       <c r="O50" s="4" t="n">
         <v>-154629135</v>
       </c>
-      <c r="P50" s="5" t="inlineStr"/>
+      <c r="P50" s="5" t="inlineStr">
+        <is>
+          <t>RevEx page 49 inferred by position (title unreadable) — verify manually</t>
+        </is>
+      </c>
       <c r="Q50" s="4" t="n">
         <v>1617446957</v>
       </c>
@@ -5649,14 +5545,12 @@
       <c r="N54" s="4" t="n">
         <v>35114726</v>
       </c>
-      <c r="O54" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="O54" s="4" t="n">
+        <v>-1414268</v>
       </c>
       <c r="P54" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: total_revenues | NOT FOUND: total_ofs</t>
+          <t>NOT FOUND: total_revenues</t>
         </is>
       </c>
       <c r="Q54" s="4" t="n">
@@ -5691,10 +5585,8 @@
       <c r="Z54" s="4" t="n">
         <v>35114726000</v>
       </c>
-      <c r="AA54" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="AA54" s="4" t="n">
+        <v>-1414268000</v>
       </c>
     </row>
     <row r="55">
@@ -6228,11 +6120,7 @@
       <c r="O60" s="4" t="n">
         <v>-595467</v>
       </c>
-      <c r="P60" s="5" t="inlineStr">
-        <is>
-          <t>BS page 60 inferred by position (title unreadable) — verify manually</t>
-        </is>
-      </c>
+      <c r="P60" s="5" t="inlineStr"/>
       <c r="Q60" s="4" t="n">
         <v>31611266000</v>
       </c>
@@ -6466,45 +6354,29 @@
           <t>Thousands</t>
         </is>
       </c>
-      <c r="E63" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="F63" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="G63" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="H63" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="I63" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="J63" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="K63" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="L63" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="E63" s="4" t="n">
+        <v>4795369</v>
+      </c>
+      <c r="F63" s="4" t="n">
+        <v>1818882</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>2645</v>
+      </c>
+      <c r="H63" s="4" t="n">
+        <v>54744</v>
+      </c>
+      <c r="I63" s="4" t="n">
+        <v>2545164</v>
+      </c>
+      <c r="J63" s="4" t="n">
+        <v>442</v>
+      </c>
+      <c r="K63" s="4" t="n">
+        <v>277171</v>
+      </c>
+      <c r="L63" s="4" t="n">
+        <v>2880166</v>
       </c>
       <c r="M63" s="4" t="n">
         <v>6308910</v>
@@ -6515,50 +6387,30 @@
       <c r="O63" s="4" t="n">
         <v>130931</v>
       </c>
-      <c r="P63" s="5" t="inlineStr">
-        <is>
-          <t>Unit disclosure differs between statement pages: {28: 'Full Dollars', 39: 'Thousands'} — verify normalized figures manually | BS p29: General Fund column not identified</t>
-        </is>
-      </c>
-      <c r="Q63" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="R63" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="S63" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="T63" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="U63" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="V63" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="W63" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="X63" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="P63" s="5" t="inlineStr"/>
+      <c r="Q63" s="4" t="n">
+        <v>4795369000</v>
+      </c>
+      <c r="R63" s="4" t="n">
+        <v>1818882000</v>
+      </c>
+      <c r="S63" s="4" t="n">
+        <v>2645000</v>
+      </c>
+      <c r="T63" s="4" t="n">
+        <v>54744000</v>
+      </c>
+      <c r="U63" s="4" t="n">
+        <v>2545164000</v>
+      </c>
+      <c r="V63" s="4" t="n">
+        <v>442000</v>
+      </c>
+      <c r="W63" s="4" t="n">
+        <v>277171000</v>
+      </c>
+      <c r="X63" s="4" t="n">
+        <v>2880166000</v>
       </c>
       <c r="Y63" s="4" t="n">
         <v>6308910000</v>
@@ -6615,26 +6467,16 @@
       <c r="L64" s="4" t="n">
         <v>1594722</v>
       </c>
-      <c r="M64" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N64" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="O64" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="P64" s="5" t="inlineStr">
-        <is>
-          <t>NOT FOUND: total_revenues | NOT FOUND: total_expenditures | NOT FOUND: total_ofs</t>
-        </is>
-      </c>
+      <c r="M64" s="4" t="n">
+        <v>6270466</v>
+      </c>
+      <c r="N64" s="4" t="n">
+        <v>6764492</v>
+      </c>
+      <c r="O64" s="4" t="n">
+        <v>161550</v>
+      </c>
+      <c r="P64" s="5" t="inlineStr"/>
       <c r="Q64" s="4" t="n">
         <v>2991167000</v>
       </c>
@@ -6659,20 +6501,14 @@
       <c r="X64" s="4" t="n">
         <v>1594722000</v>
       </c>
-      <c r="Y64" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z64" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="AA64" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="Y64" s="4" t="n">
+        <v>6270466000</v>
+      </c>
+      <c r="Z64" s="4" t="n">
+        <v>6764492000</v>
+      </c>
+      <c r="AA64" s="4" t="n">
+        <v>161550000</v>
       </c>
     </row>
     <row r="65">
@@ -7238,45 +7074,31 @@
           <t>Millions</t>
         </is>
       </c>
-      <c r="E71" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="F71" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="E71" s="4" t="n">
+        <v>89742</v>
+      </c>
+      <c r="F71" s="4" t="n">
+        <v>26969</v>
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="H71" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="I71" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="J71" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="K71" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="L71" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="H71" s="4" t="n">
+        <v>283</v>
+      </c>
+      <c r="I71" s="4" t="n">
+        <v>51745</v>
+      </c>
+      <c r="J71" s="4" t="n">
+        <v>7969</v>
+      </c>
+      <c r="K71" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="L71" s="4" t="n">
+        <v>60003</v>
       </c>
       <c r="M71" s="4" t="n">
         <v>100555</v>
@@ -7284,55 +7106,39 @@
       <c r="N71" s="4" t="n">
         <v>129020</v>
       </c>
-      <c r="O71" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="O71" s="4" t="n">
+        <v>38087</v>
       </c>
       <c r="P71" s="5" t="inlineStr">
         <is>
-          <t>Unit disclosure differs between statement pages: {16: 'Full Dollars', 43: 'Millions'} — verify normalized figures manually | BS: spread layout — General Fund column on facing page 16 | NOT FOUND: total_assets | NOT FOUND: total_liabilities | NOT FOUND: nonspendable | NOT FOUND: restricted | NOT FOUND: committed | NOT FOUND: assigned | NOT FOUND: unassigned | NOT FOUND: total_fund_balances | NOT FOUND: total_ofs</t>
-        </is>
-      </c>
-      <c r="Q71" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="R71" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+          <t>NOT FOUND: nonspendable</t>
+        </is>
+      </c>
+      <c r="Q71" s="4" t="n">
+        <v>89742000000</v>
+      </c>
+      <c r="R71" s="4" t="n">
+        <v>26969000000</v>
       </c>
       <c r="S71" s="6" t="inlineStr">
         <is>
           <t>NOT FOUND</t>
         </is>
       </c>
-      <c r="T71" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="U71" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="V71" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="W71" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="X71" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="T71" s="4" t="n">
+        <v>283000000</v>
+      </c>
+      <c r="U71" s="4" t="n">
+        <v>51745000000</v>
+      </c>
+      <c r="V71" s="4" t="n">
+        <v>7969000000</v>
+      </c>
+      <c r="W71" s="4" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="X71" s="4" t="n">
+        <v>60003000000</v>
       </c>
       <c r="Y71" s="4" t="n">
         <v>100555000000</v>
@@ -7340,10 +7146,8 @@
       <c r="Z71" s="4" t="n">
         <v>129020000000</v>
       </c>
-      <c r="AA71" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="AA71" s="4" t="n">
+        <v>38087000000</v>
       </c>
     </row>
     <row r="72">
@@ -7488,26 +7292,16 @@
       <c r="L73" s="4" t="n">
         <v>17153942</v>
       </c>
-      <c r="M73" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N73" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="O73" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="P73" s="5" t="inlineStr">
-        <is>
-          <t>Unit disclosure differs between statement pages: {45: 'Thousands', 5: 'Full Dollars'} — verify normalized figures manually | RevEx p6: General Fund column not identified</t>
-        </is>
-      </c>
+      <c r="M73" s="4" t="n">
+        <v>49343227</v>
+      </c>
+      <c r="N73" s="4" t="n">
+        <v>49447475</v>
+      </c>
+      <c r="O73" s="4" t="n">
+        <v>-520078</v>
+      </c>
+      <c r="P73" s="5" t="inlineStr"/>
       <c r="Q73" s="4" t="n">
         <v>28138624000</v>
       </c>
@@ -7532,20 +7326,14 @@
       <c r="X73" s="4" t="n">
         <v>17153942000</v>
       </c>
-      <c r="Y73" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z73" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="AA73" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="Y73" s="4" t="n">
+        <v>49343227000</v>
+      </c>
+      <c r="Z73" s="4" t="n">
+        <v>49447475000</v>
+      </c>
+      <c r="AA73" s="4" t="n">
+        <v>-520078000</v>
       </c>
     </row>
     <row r="74">
@@ -7682,26 +7470,16 @@
       <c r="L75" s="4" t="n">
         <v>179961</v>
       </c>
-      <c r="M75" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N75" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="O75" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="P75" s="5" t="inlineStr">
-        <is>
-          <t>Unit disclosure differs between statement pages: {70: 'Thousands', 69: 'Full Dollars'} — verify normalized figures manually | RevEx p70: General Fund column not identified</t>
-        </is>
-      </c>
+      <c r="M75" s="4" t="n">
+        <v>754407</v>
+      </c>
+      <c r="N75" s="4" t="n">
+        <v>721259</v>
+      </c>
+      <c r="O75" s="4" t="n">
+        <v>-26969</v>
+      </c>
+      <c r="P75" s="5" t="inlineStr"/>
       <c r="Q75" s="4" t="n">
         <v>254243000</v>
       </c>
@@ -7726,20 +7504,14 @@
       <c r="X75" s="4" t="n">
         <v>179961000</v>
       </c>
-      <c r="Y75" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z75" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="AA75" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="Y75" s="4" t="n">
+        <v>754407000</v>
+      </c>
+      <c r="Z75" s="4" t="n">
+        <v>721259000</v>
+      </c>
+      <c r="AA75" s="4" t="n">
+        <v>-26969000</v>
       </c>
     </row>
     <row r="76">
@@ -8005,14 +7777,12 @@
       <c r="N78" s="4" t="n">
         <v>94758255</v>
       </c>
-      <c r="O78" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="O78" s="4" t="n">
+        <v>-608307</v>
       </c>
       <c r="P78" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: assigned | NOT FOUND: total_ofs</t>
+          <t>NOT FOUND: assigned</t>
         </is>
       </c>
       <c r="Q78" s="4" t="n">
@@ -8047,10 +7817,8 @@
       <c r="Z78" s="4" t="n">
         <v>94758255000</v>
       </c>
-      <c r="AA78" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="AA78" s="4" t="n">
+        <v>-608307000</v>
       </c>
     </row>
     <row r="79">
@@ -8269,11 +8037,15 @@
       <c r="G81" s="4" t="n">
         <v>4964</v>
       </c>
-      <c r="H81" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I81" s="4" t="n">
-        <v>0</v>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
       </c>
       <c r="J81" s="4" t="n">
         <v>942031</v>
@@ -8290,14 +8062,12 @@
       <c r="N81" s="4" t="n">
         <v>2599721</v>
       </c>
-      <c r="O81" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="O81" s="4" t="n">
+        <v>244739</v>
       </c>
       <c r="P81" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: total_ofs</t>
+          <t>NOT FOUND: restricted | NOT FOUND: committed</t>
         </is>
       </c>
       <c r="Q81" s="4" t="n">
@@ -8309,11 +8079,15 @@
       <c r="S81" s="4" t="n">
         <v>4964000</v>
       </c>
-      <c r="T81" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U81" s="4" t="n">
-        <v>0</v>
+      <c r="T81" s="6" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
+      </c>
+      <c r="U81" s="6" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
       </c>
       <c r="V81" s="4" t="n">
         <v>942031000</v>
@@ -8330,10 +8104,8 @@
       <c r="Z81" s="4" t="n">
         <v>2599721000</v>
       </c>
-      <c r="AA81" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="AA81" s="4" t="n">
+        <v>244739000</v>
       </c>
     </row>
     <row r="82">
@@ -8844,15 +8616,11 @@
       <c r="L87" s="4" t="n">
         <v>408011072</v>
       </c>
-      <c r="M87" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N87" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="M87" s="4" t="n">
+        <v>673698004</v>
+      </c>
+      <c r="N87" s="4" t="n">
+        <v>741545891</v>
       </c>
       <c r="O87" s="3" t="inlineStr">
         <is>
@@ -8861,7 +8629,7 @@
       </c>
       <c r="P87" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: assigned | RevEx p6: General Fund column not identified</t>
+          <t>NOT FOUND: assigned | NOT FOUND: total_ofs</t>
         </is>
       </c>
       <c r="Q87" s="4" t="n">
@@ -8890,15 +8658,11 @@
       <c r="X87" s="4" t="n">
         <v>408011072</v>
       </c>
-      <c r="Y87" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z87" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="Y87" s="4" t="n">
+        <v>673698004</v>
+      </c>
+      <c r="Z87" s="4" t="n">
+        <v>741545891</v>
       </c>
       <c r="AA87" s="6" t="inlineStr">
         <is>
@@ -9294,7 +9058,7 @@
         </is>
       </c>
       <c r="G92" s="4" t="n">
-        <v>-16534469</v>
+        <v>2101250</v>
       </c>
       <c r="H92" s="4" t="n">
         <v>4646911</v>
@@ -9342,7 +9106,7 @@
         </is>
       </c>
       <c r="S92" s="4" t="n">
-        <v>-16534469</v>
+        <v>2101250</v>
       </c>
       <c r="T92" s="4" t="n">
         <v>4646911</v>
@@ -9611,7 +9375,7 @@
       </c>
       <c r="P95" s="5" t="inlineStr">
         <is>
-          <t>BS page 46 inferred by position (title unreadable) — verify manually | NOT FOUND: unassigned</t>
+          <t>NOT FOUND: unassigned</t>
         </is>
       </c>
       <c r="Q95" s="4" t="n">

</xml_diff>

<commit_message>
Results: band refinement — 1044/1100 (94.9%), 3 shipped values corrected
- Coverage 1033 -> 1044; identity audit 0 findings (FB 79/79 all sets)
- All 16 changed cells adjudicated: Mesa +3, Salt Lake +5 (verified
  truths), Pima/Ada/Bexar/Kentucky bonuses, Louisville honesty
  conversion, and three CORRECTIONS to previously shipped values
  (Oakland fabricated digit, Massachusetts deferred-inflows line,
  Montgomery missed -421.6M OFS) — each re-derived from the PDF
- Texas regression from the interim run fixed and held
- Backup refreshed; docs updated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Backups/2026-07-07_audited/FY25_Set3_results.xlsx
+++ b/Backups/2026-07-07_audited/FY25_Set3_results.xlsx
@@ -1029,26 +1029,16 @@
       <c r="L6" s="4" t="n">
         <v>438993</v>
       </c>
-      <c r="M6" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N6" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="O6" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="P6" s="5" t="inlineStr">
-        <is>
-          <t>NOT FOUND: total_revenues | NOT FOUND: total_expenditures | NOT FOUND: total_ofs</t>
-        </is>
-      </c>
+      <c r="M6" s="4" t="n">
+        <v>571994</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>625809</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>70076</v>
+      </c>
+      <c r="P6" s="5" t="inlineStr"/>
       <c r="Q6" s="4" t="n">
         <v>531566000</v>
       </c>
@@ -1073,20 +1063,14 @@
       <c r="X6" s="4" t="n">
         <v>438993000</v>
       </c>
-      <c r="Y6" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z6" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="AA6" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="Y6" s="4" t="n">
+        <v>571994000</v>
+      </c>
+      <c r="Z6" s="4" t="n">
+        <v>625809000</v>
+      </c>
+      <c r="AA6" s="4" t="n">
+        <v>70076000</v>
       </c>
     </row>
     <row r="7">
@@ -1303,10 +1287,8 @@
       <c r="E9" s="4" t="n">
         <v>259595</v>
       </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="F9" s="4" t="n">
+        <v>41206</v>
       </c>
       <c r="G9" s="4" t="n">
         <v>2851</v>
@@ -1339,16 +1321,14 @@
       </c>
       <c r="P9" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: total_liabilities | NOT FOUND: restricted</t>
+          <t>NOT FOUND: restricted</t>
         </is>
       </c>
       <c r="Q9" s="4" t="n">
         <v>259595000</v>
       </c>
-      <c r="R9" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="R9" s="4" t="n">
+        <v>41206000</v>
       </c>
       <c r="S9" s="4" t="n">
         <v>2851000</v>
@@ -3375,7 +3355,7 @@
       </c>
       <c r="P31" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: nonspendable | OFS total found via positional fallback (label non-standard)</t>
+          <t>NOT FOUND: nonspendable</t>
         </is>
       </c>
       <c r="Q31" s="4" t="n">
@@ -3636,10 +3616,8 @@
       <c r="E34" s="4" t="n">
         <v>335249913</v>
       </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="F34" s="4" t="n">
+        <v>49746391</v>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
@@ -3674,16 +3652,14 @@
       </c>
       <c r="P34" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: total_liabilities | NOT FOUND: nonspendable | NOT FOUND: committed</t>
+          <t>NOT FOUND: nonspendable | NOT FOUND: committed</t>
         </is>
       </c>
       <c r="Q34" s="4" t="n">
         <v>335249913</v>
       </c>
-      <c r="R34" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="R34" s="4" t="n">
+        <v>49746391</v>
       </c>
       <c r="S34" s="6" t="inlineStr">
         <is>
@@ -4313,8 +4289,10 @@
       <c r="G41" s="4" t="n">
         <v>7407957</v>
       </c>
-      <c r="H41" s="4" t="n">
-        <v>0</v>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
       </c>
       <c r="I41" s="4" t="n">
         <v>105155555</v>
@@ -4337,7 +4315,11 @@
       <c r="O41" s="4" t="n">
         <v>-98995629</v>
       </c>
-      <c r="P41" s="5" t="inlineStr"/>
+      <c r="P41" s="5" t="inlineStr">
+        <is>
+          <t>NOT FOUND: restricted</t>
+        </is>
+      </c>
       <c r="Q41" s="4" t="n">
         <v>301157079</v>
       </c>
@@ -4347,8 +4329,10 @@
       <c r="S41" s="4" t="n">
         <v>7407957</v>
       </c>
-      <c r="T41" s="4" t="n">
-        <v>0</v>
+      <c r="T41" s="6" t="inlineStr">
+        <is>
+          <t>NOT FOUND</t>
+        </is>
       </c>
       <c r="U41" s="4" t="n">
         <v>105155555</v>
@@ -4402,10 +4386,8 @@
       <c r="G42" s="4" t="n">
         <v>6485</v>
       </c>
-      <c r="H42" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="H42" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="I42" s="4" t="n">
         <v>0</v>
@@ -4428,11 +4410,7 @@
       <c r="O42" s="4" t="n">
         <v>-1320063</v>
       </c>
-      <c r="P42" s="5" t="inlineStr">
-        <is>
-          <t>NOT FOUND: restricted</t>
-        </is>
-      </c>
+      <c r="P42" s="5" t="inlineStr"/>
       <c r="Q42" s="4" t="n">
         <v>8047275000</v>
       </c>
@@ -4442,10 +4420,8 @@
       <c r="S42" s="4" t="n">
         <v>6485000</v>
       </c>
-      <c r="T42" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="T42" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="U42" s="4" t="n">
         <v>0</v>
@@ -4680,7 +4656,7 @@
         <v>20222751</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>7380974</v>
+        <v>6681314</v>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
@@ -4715,14 +4691,14 @@
       </c>
       <c r="P45" s="5" t="inlineStr">
         <is>
-          <t>BS p55: continuation carries other funds — page skipped | NOT FOUND: nonspendable | NOT FOUND: total_fund_balances | RevEx re-extracted via OCR (native value zone unreadable) — verify manually</t>
+          <t>BS p55: continuation carries other funds — page skipped | NOT FOUND: nonspendable | NOT FOUND: total_fund_balances</t>
         </is>
       </c>
       <c r="Q45" s="4" t="n">
         <v>20222751000</v>
       </c>
       <c r="R45" s="4" t="n">
-        <v>7380974000</v>
+        <v>6681314000</v>
       </c>
       <c r="S45" s="6" t="inlineStr">
         <is>
@@ -4905,13 +4881,9 @@
         <v>4034468463</v>
       </c>
       <c r="O47" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P47" s="5" t="inlineStr">
-        <is>
-          <t>RevEx p57: continuation carries other funds — page skipped | OFS total found via positional fallback (label non-standard)</t>
-        </is>
-      </c>
+        <v>-421590235</v>
+      </c>
+      <c r="P47" s="5" t="inlineStr"/>
       <c r="Q47" s="4" t="n">
         <v>1986863035</v>
       </c>
@@ -4943,7 +4915,7 @@
         <v>4034468463</v>
       </c>
       <c r="AA47" s="4" t="n">
-        <v>0</v>
+        <v>-421590235</v>
       </c>
     </row>
     <row r="48">
@@ -5247,7 +5219,7 @@
         </is>
       </c>
       <c r="E51" s="4" t="n">
-        <v>3561941373</v>
+        <v>356194137</v>
       </c>
       <c r="F51" s="4" t="n">
         <v>66260526</v>
@@ -5281,7 +5253,7 @@
       </c>
       <c r="P51" s="5" t="inlineStr"/>
       <c r="Q51" s="4" t="n">
-        <v>3561941373</v>
+        <v>356194137</v>
       </c>
       <c r="R51" s="4" t="n">
         <v>66260526</v>
@@ -8622,14 +8594,12 @@
       <c r="N87" s="4" t="n">
         <v>741545891</v>
       </c>
-      <c r="O87" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="O87" s="4" t="n">
+        <v>172185393</v>
       </c>
       <c r="P87" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: assigned | NOT FOUND: total_ofs</t>
+          <t>NOT FOUND: assigned</t>
         </is>
       </c>
       <c r="Q87" s="4" t="n">
@@ -8664,10 +8634,8 @@
       <c r="Z87" s="4" t="n">
         <v>741545891</v>
       </c>
-      <c r="AA87" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="AA87" s="4" t="n">
+        <v>172185393</v>
       </c>
     </row>
     <row r="88">
@@ -9047,15 +9015,11 @@
           <t>Full Dollars</t>
         </is>
       </c>
-      <c r="E92" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="F92" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="E92" s="4" t="n">
+        <v>352936444</v>
+      </c>
+      <c r="F92" s="4" t="n">
+        <v>30709428</v>
       </c>
       <c r="G92" s="4" t="n">
         <v>2101250</v>
@@ -9072,38 +9036,24 @@
       <c r="K92" s="4" t="n">
         <v>148841970</v>
       </c>
-      <c r="L92" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="M92" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N92" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="L92" s="4" t="n">
+        <v>316901400</v>
+      </c>
+      <c r="M92" s="4" t="n">
+        <v>471584793</v>
+      </c>
+      <c r="N92" s="4" t="n">
+        <v>466532282</v>
       </c>
       <c r="O92" s="4" t="n">
         <v>37337553</v>
       </c>
-      <c r="P92" s="5" t="inlineStr">
-        <is>
-          <t>NOT FOUND: total_assets | NOT FOUND: total_liabilities | NOT FOUND: total_fund_balances | NOT FOUND: total_revenues | NOT FOUND: total_expenditures</t>
-        </is>
-      </c>
-      <c r="Q92" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="R92" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="P92" s="5" t="inlineStr"/>
+      <c r="Q92" s="4" t="n">
+        <v>352936444</v>
+      </c>
+      <c r="R92" s="4" t="n">
+        <v>30709428</v>
       </c>
       <c r="S92" s="4" t="n">
         <v>2101250</v>
@@ -9120,20 +9070,14 @@
       <c r="W92" s="4" t="n">
         <v>148841970</v>
       </c>
-      <c r="X92" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Y92" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z92" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="X92" s="4" t="n">
+        <v>316901400</v>
+      </c>
+      <c r="Y92" s="4" t="n">
+        <v>471584793</v>
+      </c>
+      <c r="Z92" s="4" t="n">
+        <v>466532282</v>
       </c>
       <c r="AA92" s="4" t="n">
         <v>37337553</v>

</xml_diff>

<commit_message>
Results: Honolulu wave — 1049/1100 (95.4%), audit clean
- Coverage 1044 -> 1049; 5 changed cells, ALL gains (Honolulu +4 with
  verified truth values, Kansas City OFS bonus from compact matching)
- Identity audit: 0 findings, FB identity 79/79 across all three sets
- Backup refreshed; docs updated

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Backups/2026-07-07_audited/FY25_Set3_results.xlsx
+++ b/Backups/2026-07-07_audited/FY25_Set3_results.xlsx
@@ -3201,10 +3201,8 @@
           <t>Thousands</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="E30" s="4" t="n">
+        <v>1252166</v>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
@@ -3231,30 +3229,22 @@
       <c r="L30" s="4" t="n">
         <v>967491</v>
       </c>
-      <c r="M30" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="N30" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="O30" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="M30" s="4" t="n">
+        <v>2088725</v>
+      </c>
+      <c r="N30" s="4" t="n">
+        <v>1519815</v>
+      </c>
+      <c r="O30" s="4" t="n">
+        <v>-480436</v>
       </c>
       <c r="P30" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: total_assets | NOT FOUND: total_liabilities | NOT FOUND: nonspendable | RevEx p70: continuation carries other funds — page skipped | NOT FOUND: total_revenues | NOT FOUND: total_expenditures | NOT FOUND: total_ofs</t>
-        </is>
-      </c>
-      <c r="Q30" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+          <t>NOT FOUND: total_liabilities | NOT FOUND: nonspendable</t>
+        </is>
+      </c>
+      <c r="Q30" s="4" t="n">
+        <v>1252166000</v>
       </c>
       <c r="R30" s="6" t="inlineStr">
         <is>
@@ -3281,20 +3271,14 @@
       <c r="X30" s="4" t="n">
         <v>967491000</v>
       </c>
-      <c r="Y30" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="Z30" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
-      </c>
-      <c r="AA30" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="Y30" s="4" t="n">
+        <v>2088725000</v>
+      </c>
+      <c r="Z30" s="4" t="n">
+        <v>1519815000</v>
+      </c>
+      <c r="AA30" s="4" t="n">
+        <v>-480436000</v>
       </c>
     </row>
     <row r="31">
@@ -5614,14 +5598,12 @@
       <c r="N55" s="4" t="n">
         <v>711441</v>
       </c>
-      <c r="O55" s="3" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="O55" s="4" t="n">
+        <v>-51906</v>
       </c>
       <c r="P55" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: nonspendable | NOT FOUND: total_ofs</t>
+          <t>NOT FOUND: nonspendable</t>
         </is>
       </c>
       <c r="Q55" s="4" t="n">
@@ -5656,10 +5638,8 @@
       <c r="Z55" s="4" t="n">
         <v>711441000</v>
       </c>
-      <c r="AA55" s="6" t="inlineStr">
-        <is>
-          <t>NOT FOUND</t>
-        </is>
+      <c r="AA55" s="4" t="n">
+        <v>-51906000</v>
       </c>
     </row>
     <row r="56">
@@ -7645,7 +7625,7 @@
       </c>
       <c r="P77" s="5" t="inlineStr">
         <is>
-          <t>NOT FOUND: nonspendable | NOT FOUND: restricted | NOT FOUND: committed | NOT FOUND: assigned | NOT FOUND: unassigned | NOT FOUND: total_fund_balances | RevEx re-extracted via OCR (native value zone unreadable) — verify manually | NOT FOUND: total_ofs</t>
+          <t>NOT FOUND: nonspendable | NOT FOUND: restricted | NOT FOUND: committed | NOT FOUND: assigned | NOT FOUND: unassigned | NOT FOUND: total_fund_balances | NOT FOUND: total_ofs</t>
         </is>
       </c>
       <c r="Q77" s="4" t="n">

</xml_diff>